<commit_message>
Actualiza closet con marco posterior completo sin panel
</commit_message>
<xml_diff>
--- a/compras-proyecto.xlsx
+++ b/compras-proyecto.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resumen" sheetId="1" r:id="Rb3cf6cb0595742d6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pedido de corte" sheetId="2" r:id="R9f55693a104b43ca"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Láminas" sheetId="3" r:id="Rf5fef9e5deff44b5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cantos" sheetId="4" r:id="R5736bd6e5b5c4ea1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Compras" sheetId="5" r:id="R2332c494379743bd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bloqueos" sheetId="6" r:id="R26475d8f3f5140dc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="En el armado" sheetId="7" r:id="Rc249f97e798842ad"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resumen" sheetId="1" r:id="R22261d597eb64c5e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pedido de corte" sheetId="2" r:id="R1aee4edc6ec641ea"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Láminas" sheetId="3" r:id="R5cdc49ae4d094ad2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cantos" sheetId="4" r:id="R9f55a881f64e4ed8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Compras" sheetId="5" r:id="R89e54929ecef4b62"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bloqueos" sheetId="6" r:id="Rd41c2da8a27c4626"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="En el armado" sheetId="7" r:id="R87b8fa41abe74842"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -405,7 +405,7 @@
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="11" t="str">
-        <x:v>Estimación conjunta del 27/10/2026, generada desde los Excel de cada mueble (herramientas/build_compras_proyecto.py).</x:v>
+        <x:v>Estimación conjunta del 28/10/2026, generada desde los Excel de cada mueble (herramientas/build_compras_proyecto.py).</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
@@ -427,13 +427,13 @@
         <x:v>Láminas RH15</x:v>
       </x:c>
       <x:c r="B7" s="13" t="n">
-        <x:v>10</x:v>
+        <x:v>9</x:v>
       </x:c>
       <x:c r="C7" s="13" t="n">
         <x:v>8</x:v>
       </x:c>
       <x:c r="D7" s="13" t="str">
-        <x:v>Cocina 4 + clóset 5 + baño 1 por separado; encaje conjunto en la hoja Láminas.</x:v>
+        <x:v>Cocina 4 + clóset 4 + baño 1 por separado; encaje conjunto en la hoja Láminas.</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
@@ -475,7 +475,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="D10" s="13" t="str">
-        <x:v>Sobran unos 28 m para cantear piezas pequeñas en el armado.</x:v>
+        <x:v>Sobran unos 19 m para cantear piezas pequeñas en el armado.</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
@@ -753,7 +753,7 @@
         <v>150 × 99,1</v>
       </c>
       <c r="P9" s="17" t="str">
-        <v>Si no la cantean: cortar a 150 × 99.1 y cantear en el armado. Rebaje para la gola en el armado, cuando se defina el borde del granito; no lo hace el proveedor.</v>
+        <v>Si no la cantean: cortar a 150 × 99,1 y cantear en el armado. Rebaje para la gola en el armado, cuando se defina el borde del granito; no lo hace el proveedor.</v>
       </c>
     </row>
     <row r="10">
@@ -1003,7 +1003,7 @@
         <v>570 × 99,55</v>
       </c>
       <c r="P14" s="17" t="str">
-        <v>Si no la cantean: cortar a 570 × 99.55 y cantear en el armado.</v>
+        <v>Si no la cantean: cortar a 570 × 99,55 y cantear en el armado.</v>
       </c>
     </row>
     <row r="15" ht="28.799999237060547">
@@ -1103,7 +1103,7 @@
         <v>570 × 79,55</v>
       </c>
       <c r="P16" s="17" t="str">
-        <v>Si no la cantean: cortar a 570 × 79.55 y cantear en el armado.</v>
+        <v>Si no la cantean: cortar a 570 × 79,55 y cantear en el armado.</v>
       </c>
     </row>
     <row r="17" ht="43.20000076293945">
@@ -1303,7 +1303,7 @@
         <v>640 × 99,1</v>
       </c>
       <c r="P20" s="17" t="str">
-        <v>Si no la cantean: cortar a 640 × 99.1 y cantear en el armado. Rebaje para la gola en el armado, cuando se defina el borde del granito; no lo hace el proveedor.</v>
+        <v>Si no la cantean: cortar a 640 × 99,1 y cantear en el armado. Rebaje para la gola en el armado, cuando se defina el borde del granito; no lo hace el proveedor.</v>
       </c>
     </row>
     <row r="21">
@@ -1503,7 +1503,7 @@
         <v>549,55 × 74,55</v>
       </c>
       <c r="P24" s="17" t="str">
-        <v>Si no la cantean: cortar a 549.55 × 74.55 y cantear en el armado.</v>
+        <v>Si no la cantean: cortar a 549,55 × 74,55 y cantear en el armado.</v>
       </c>
     </row>
     <row r="25">
@@ -1553,7 +1553,7 @@
         <v>583 × 74,55</v>
       </c>
       <c r="P25" s="17" t="str">
-        <v>Si no la cantean: cortar a 583 × 74.55 y cantear en el armado.</v>
+        <v>Si no la cantean: cortar a 583 × 74,55 y cantear en el armado.</v>
       </c>
     </row>
     <row r="26">
@@ -1853,7 +1853,7 @@
         <v>669,1 × 99,1</v>
       </c>
       <c r="P31" s="17" t="str">
-        <v>Si no la cantean: cortar a 669.1 × 99.1 y cantear en el armado. Rebaje para la gola en el armado, cuando se defina el borde del granito; no lo hace el proveedor.</v>
+        <v>Si no la cantean: cortar a 669,1 × 99,1 y cantear en el armado. Rebaje para la gola en el armado, cuando se defina el borde del granito; no lo hace el proveedor.</v>
       </c>
     </row>
     <row r="32">
@@ -2203,7 +2203,7 @@
         <v>370 × 99,1</v>
       </c>
       <c r="P38" s="17" t="str">
-        <v>Si no la cantean: cortar a 370 × 99.1 y cantear en el armado. Rebaje para la gola en el armado, cuando se defina el borde del granito; no lo hace el proveedor.</v>
+        <v>Si no la cantean: cortar a 370 × 99,1 y cantear en el armado. Rebaje para la gola en el armado, cuando se defina el borde del granito; no lo hace el proveedor.</v>
       </c>
     </row>
     <row r="39">
@@ -2503,7 +2503,7 @@
         <v>1274,1 × 96,1</v>
       </c>
       <c r="P44" s="17" t="str">
-        <v>Si no la cantean: cortar a 1274.1 × 96.1 y cantear en el armado.</v>
+        <v>Si no la cantean: cortar a 1274,1 × 96,1 y cantear en el armado.</v>
       </c>
     </row>
     <row r="45">
@@ -3103,7 +3103,7 @@
         <v>569,1 × 59,1</v>
       </c>
       <c r="P56" s="17" t="str">
-        <v>Si no la cantean: cortar a 569.1 × 59.1 y cantear en el armado. P071: flexible 0,45 mm en los cuatro bordes. Confirmar cabida en canteadora; si la rechaza, cantear en taller con el descuento correspondiente.</v>
+        <v>Si no la cantean: cortar a 569,1 × 59,1 y cantear en el armado. P071: flexible 0,45 mm en los cuatro bordes. Confirmar cabida en canteadora; si la rechaza, cantear en taller con el descuento correspondiente.</v>
       </c>
     </row>
     <row r="57">
@@ -3447,7 +3447,7 @@
         <v>Normal</v>
       </c>
       <c r="N63" s="16" t="str">
-        <v>717 × 324.5</v>
+        <v>717 × 324,5</v>
       </c>
       <c r="O63" s="16" t="str">
         <v>713 × 320,5</v>
@@ -3497,7 +3497,7 @@
         <v>Normal</v>
       </c>
       <c r="N64" s="16" t="str">
-        <v>717 × 324.5</v>
+        <v>717 × 324,5</v>
       </c>
       <c r="O64" s="16" t="str">
         <v>713 × 320,5</v>
@@ -3653,7 +3653,7 @@
         <v>684,1 × 59,1</v>
       </c>
       <c r="P67" s="17" t="str">
-        <v>Si no la cantean: cortar a 684.1 × 59.1 y cantear en el armado.</v>
+        <v>Si no la cantean: cortar a 684,1 × 59,1 y cantear en el armado.</v>
       </c>
     </row>
     <row r="68">
@@ -3703,7 +3703,7 @@
         <v>684,1 × 79,1</v>
       </c>
       <c r="P68" s="17" t="str">
-        <v>Si no la cantean: cortar a 684.1 × 79.1 y cantear en el armado.</v>
+        <v>Si no la cantean: cortar a 684,1 × 79,1 y cantear en el armado.</v>
       </c>
     </row>
     <row r="69">
@@ -3797,7 +3797,7 @@
         <v>Normal</v>
       </c>
       <c r="N70" s="16" t="str">
-        <v>717 × 354.5</v>
+        <v>717 × 354,5</v>
       </c>
       <c r="O70" s="16" t="str">
         <v>713 × 350,5</v>
@@ -3847,7 +3847,7 @@
         <v>Normal</v>
       </c>
       <c r="N71" s="16" t="str">
-        <v>717 × 354.5</v>
+        <v>717 × 354,5</v>
       </c>
       <c r="O71" s="16" t="str">
         <v>713 × 350,5</v>
@@ -4361,13 +4361,13 @@
         <v>Clóset</v>
       </c>
       <c r="B82" s="16" t="str">
-        <v>C3-005</v>
+        <v>C3-025</v>
       </c>
       <c r="C82" s="16" t="str">
         <v>B1</v>
       </c>
       <c r="D82" s="17" t="str">
-        <v>Fondo RH15</v>
+        <v>Amarre posterior superior izquierdo</v>
       </c>
       <c r="E82" s="16" t="str">
         <v>RH15 Cartagena 15 mm</v>
@@ -4376,13 +4376,13 @@
         <v>1</v>
       </c>
       <c r="G82" s="16" t="n">
-        <v>2250</v>
+        <v>830</v>
       </c>
       <c r="H82" s="16" t="n">
-        <v>830</v>
+        <v>100</v>
       </c>
       <c r="I82" s="16" t="str">
-        <v>—</v>
+        <v>F</v>
       </c>
       <c r="J82" s="16" t="str">
         <v>—</v>
@@ -4394,16 +4394,16 @@
         <v>—</v>
       </c>
       <c r="M82" s="16" t="str">
-        <v>Sin canto</v>
+        <v>Pequeña</v>
       </c>
       <c r="N82" s="16" t="str">
-        <v>2250 × 830</v>
+        <v>830 × 100</v>
       </c>
       <c r="O82" s="16" t="str">
-        <v>2250 × 830</v>
+        <v>830 × 99,55</v>
       </c>
       <c r="P82" s="17" t="str">
-        <v>—</v>
+        <v>Si no la cantean: cortar a 830 × 99.55 y cantear en el armado. Marco posterior RH15 sin panel de fondo. Flexible 0,45 mm solo en el borde largo inferior libre hacia el interior; los otros tres bordes son uniones ocultas sin canto. Unir a la caja y al resto del marco. Anclajes al muro posterior resistente y al izquierdo por dimensionar; no fijar solo al estuco.</v>
       </c>
     </row>
     <row r="83">
@@ -4661,13 +4661,13 @@
         <v>Clóset</v>
       </c>
       <c r="B88" s="16" t="str">
-        <v>C3-011</v>
+        <v>C3-026</v>
       </c>
       <c r="C88" s="16" t="str">
         <v>B2</v>
       </c>
       <c r="D88" s="17" t="str">
-        <v>Fondo RH15</v>
+        <v>Amarre posterior superior derecho</v>
       </c>
       <c r="E88" s="16" t="str">
         <v>RH15 Cartagena 15 mm</v>
@@ -4676,13 +4676,13 @@
         <v>1</v>
       </c>
       <c r="G88" s="16" t="n">
-        <v>2250</v>
+        <v>1075</v>
       </c>
       <c r="H88" s="16" t="n">
-        <v>1075</v>
+        <v>100</v>
       </c>
       <c r="I88" s="16" t="str">
-        <v>—</v>
+        <v>F</v>
       </c>
       <c r="J88" s="16" t="str">
         <v>—</v>
@@ -4694,16 +4694,16 @@
         <v>—</v>
       </c>
       <c r="M88" s="16" t="str">
-        <v>Sin canto</v>
+        <v>Pequeña</v>
       </c>
       <c r="N88" s="16" t="str">
-        <v>2250 × 1075</v>
+        <v>1075 × 100</v>
       </c>
       <c r="O88" s="16" t="str">
-        <v>2250 × 1075</v>
+        <v>1075 × 99,55</v>
       </c>
       <c r="P88" s="17" t="str">
-        <v>—</v>
+        <v>Si no la cantean: cortar a 1075 × 99.55 y cantear en el armado. Marco posterior RH15 sin panel de fondo. Flexible 0,45 mm solo en el borde largo inferior libre hacia el interior; los otros tres bordes son uniones ocultas sin canto. Unir a la caja y al resto del marco. Anclajes al muro posterior resistente y al izquierdo por dimensionar; no fijar solo al estuco.</v>
       </c>
     </row>
     <row r="89">
@@ -5358,202 +5358,202 @@
     </row>
     <row r="102" ht="28.799999237060547">
       <c r="A102" s="16" t="str">
-        <v>Baño</v>
+        <v>Clóset</v>
       </c>
       <c r="B102" s="16" t="str">
-        <v>B01</v>
+        <v>C3-027</v>
       </c>
       <c r="C102" s="16" t="str">
-        <v>BAJO</v>
+        <v>B2</v>
       </c>
       <c r="D102" s="17" t="str">
-        <v>Lateral</v>
+        <v>Montante posterior derecho</v>
       </c>
       <c r="E102" s="16" t="str">
-        <v>RH15 Cartagena</v>
+        <v>RH15 Cartagena 15 mm</v>
       </c>
       <c r="F102" s="16" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G102" s="16" t="n">
-        <v>470</v>
+        <v>2050</v>
       </c>
       <c r="H102" s="16" t="n">
-        <v>450</v>
+        <v>100</v>
       </c>
       <c r="I102" s="16" t="str">
         <v>F</v>
       </c>
       <c r="J102" s="16" t="str">
-        <v>F</v>
+        <v>—</v>
       </c>
       <c r="K102" s="16" t="str">
-        <v>F</v>
+        <v>—</v>
       </c>
       <c r="L102" s="16" t="str">
-        <v>F</v>
+        <v>—</v>
       </c>
       <c r="M102" s="16" t="str">
-        <v>Normal</v>
+        <v>Pequeña</v>
       </c>
       <c r="N102" s="16" t="str">
-        <v>470 × 450</v>
+        <v>2050 × 100</v>
       </c>
       <c r="O102" s="16" t="str">
-        <v>469,1 × 449,1</v>
+        <v>2050 × 99,55</v>
       </c>
       <c r="P102" s="17" t="str">
-        <v>Zona húmeda: proteger todos los bordes y sellar perforaciones; dimensiones terminadas. Canto flexible 0,45 mm en todo el perímetro; mantener sellados recortes y perforaciones.</v>
+        <v>Si no la cantean: cortar a 2050 × 99.55 y cantear en el armado. Marco posterior RH15 sin panel de fondo. Flexible 0,45 mm solo en el borde largo izquierdo libre hacia el interior; los otros tres bordes son uniones ocultas sin canto. Unir a la caja y al resto del marco. Anclajes al muro posterior resistente y al izquierdo por dimensionar; no fijar solo al estuco.</v>
       </c>
     </row>
     <row r="103" ht="28.799999237060547">
       <c r="A103" s="16" t="str">
-        <v>Baño</v>
+        <v>Clóset</v>
       </c>
       <c r="B103" s="16" t="str">
-        <v>B02</v>
+        <v>C3-028</v>
       </c>
       <c r="C103" s="16" t="str">
-        <v>BAJO</v>
+        <v>B1</v>
       </c>
       <c r="D103" s="17" t="str">
-        <v>Piso</v>
+        <v>Montante posterior izquierdo</v>
       </c>
       <c r="E103" s="16" t="str">
-        <v>RH15 Cartagena</v>
+        <v>RH15 Cartagena 15 mm</v>
       </c>
       <c r="F103" s="16" t="n">
         <v>1</v>
       </c>
       <c r="G103" s="16" t="n">
-        <v>490</v>
+        <v>2050</v>
       </c>
       <c r="H103" s="16" t="n">
-        <v>450</v>
+        <v>100</v>
       </c>
       <c r="I103" s="16" t="str">
         <v>F</v>
       </c>
       <c r="J103" s="16" t="str">
-        <v>F</v>
+        <v>—</v>
       </c>
       <c r="K103" s="16" t="str">
-        <v>F</v>
+        <v>—</v>
       </c>
       <c r="L103" s="16" t="str">
-        <v>F</v>
+        <v>—</v>
       </c>
       <c r="M103" s="16" t="str">
-        <v>Normal</v>
+        <v>Pequeña</v>
       </c>
       <c r="N103" s="16" t="str">
-        <v>490 × 450</v>
+        <v>2050 × 100</v>
       </c>
       <c r="O103" s="16" t="str">
-        <v>489,1 × 449,1</v>
+        <v>2050 × 99,55</v>
       </c>
       <c r="P103" s="17" t="str">
-        <v>Zona húmeda: proteger todos los bordes y sellar perforaciones; dimensiones terminadas. Canto flexible 0,45 mm en todo el perímetro; mantener sellados recortes y perforaciones.</v>
+        <v>Si no la cantean: cortar a 2050 × 99.55 y cantear en el armado. Marco posterior RH15 sin panel de fondo. Flexible 0,45 mm solo en el borde largo derecho libre hacia el interior; los otros tres bordes son uniones ocultas sin canto. Unir a la caja y al resto del marco. Anclajes al muro posterior resistente y al izquierdo por dimensionar; no fijar solo al estuco.</v>
       </c>
     </row>
     <row r="104" ht="57.599998474121094">
       <c r="A104" s="16" t="str">
-        <v>Baño</v>
+        <v>Clóset</v>
       </c>
       <c r="B104" s="16" t="str">
-        <v>B03</v>
+        <v>C3-029</v>
       </c>
       <c r="C104" s="16" t="str">
-        <v>BAJO</v>
+        <v>B1</v>
       </c>
       <c r="D104" s="17" t="str">
-        <v>Entrepaño retranqueado con reserva de sifón</v>
+        <v>Amarre posterior inferior izquierdo</v>
       </c>
       <c r="E104" s="16" t="str">
-        <v>RH15 Cartagena</v>
+        <v>RH15 Cartagena 15 mm</v>
       </c>
       <c r="F104" s="16" t="n">
         <v>1</v>
       </c>
       <c r="G104" s="16" t="n">
-        <v>490</v>
+        <v>830</v>
       </c>
       <c r="H104" s="16" t="n">
-        <v>405</v>
+        <v>100</v>
       </c>
       <c r="I104" s="16" t="str">
         <v>F</v>
       </c>
       <c r="J104" s="16" t="str">
-        <v>F</v>
+        <v>—</v>
       </c>
       <c r="K104" s="16" t="str">
-        <v>F</v>
+        <v>—</v>
       </c>
       <c r="L104" s="16" t="str">
-        <v>F</v>
+        <v>—</v>
       </c>
       <c r="M104" s="16" t="str">
-        <v>Normal</v>
+        <v>Pequeña</v>
       </c>
       <c r="N104" s="16" t="str">
-        <v>490 × 405</v>
+        <v>830 × 100</v>
       </c>
       <c r="O104" s="16" t="str">
-        <v>489,1 × 404,1</v>
+        <v>830 × 99,55</v>
       </c>
       <c r="P104" s="17" t="str">
-        <v>Zona húmeda: proteger todos los bordes y sellar perforaciones; dimensiones terminadas. Nicho libre de 150 mm bajo granito. Recorte trasero ilustrativo 100 × 270 mm, centrado; no mecanizar sin sifón real. Retranqueo frontal de 30 mm para agarre. Canto flexible 0,45 mm en todo el perímetro; mantener sellados recortes y perforaciones.</v>
+        <v>Si no la cantean: cortar a 830 × 99.55 y cantear en el armado. Marco posterior RH15 sin panel de fondo. Flexible 0,45 mm solo en el borde largo superior libre hacia el interior; los otros tres bordes son uniones ocultas sin canto. Unir a la caja y al resto del marco. Anclajes al muro posterior resistente y al izquierdo por dimensionar; no fijar solo al estuco.</v>
       </c>
     </row>
     <row r="105" ht="57.599998474121094">
       <c r="A105" s="16" t="str">
-        <v>Baño</v>
+        <v>Clóset</v>
       </c>
       <c r="B105" s="16" t="str">
-        <v>B04</v>
+        <v>C3-030</v>
       </c>
       <c r="C105" s="16" t="str">
-        <v>BAJO</v>
+        <v>B2</v>
       </c>
       <c r="D105" s="17" t="str">
-        <v>Travesaño trasero superior lateral</v>
+        <v>Amarre posterior inferior derecho</v>
       </c>
       <c r="E105" s="16" t="str">
-        <v>RH15 Cartagena</v>
+        <v>RH15 Cartagena 15 mm</v>
       </c>
       <c r="F105" s="16" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G105" s="16" t="n">
-        <v>195</v>
+        <v>1075</v>
       </c>
       <c r="H105" s="16" t="n">
-        <v>80</v>
+        <v>100</v>
       </c>
       <c r="I105" s="16" t="str">
         <v>F</v>
       </c>
       <c r="J105" s="16" t="str">
-        <v>F</v>
+        <v>—</v>
       </c>
       <c r="K105" s="16" t="str">
-        <v>F</v>
+        <v>—</v>
       </c>
       <c r="L105" s="16" t="str">
-        <v>F</v>
+        <v>—</v>
       </c>
       <c r="M105" s="16" t="str">
         <v>Pequeña</v>
       </c>
       <c r="N105" s="16" t="str">
-        <v>195 × 80</v>
+        <v>1075 × 100</v>
       </c>
       <c r="O105" s="16" t="str">
-        <v>194,1 × 79,1</v>
+        <v>1075 × 99,55</v>
       </c>
       <c r="P105" s="17" t="str">
-        <v>Si no la cantean: cortar a 194.1 × 79.1 y cantear en taller. Zona húmeda: proteger todos los bordes y sellar perforaciones; dimensiones terminadas. De canto, interrumpido en el centro para tuberías; no es un colgador certificado. Canto flexible 0,45 mm en todo el perímetro; mantener sellados recortes y perforaciones.</v>
+        <v>Si no la cantean: cortar a 1075 × 99.55 y cantear en el armado. Marco posterior RH15 sin panel de fondo. Flexible 0,45 mm solo en el borde largo superior libre hacia el interior; los otros tres bordes son uniones ocultas sin canto. Unir a la caja y al resto del marco. Anclajes al muro posterior resistente y al izquierdo por dimensionar; no fijar solo al estuco.</v>
       </c>
     </row>
     <row r="106" ht="57.599998474121094">
@@ -5561,25 +5561,25 @@
         <v>Baño</v>
       </c>
       <c r="B106" s="16" t="str">
-        <v>B05</v>
+        <v>B01</v>
       </c>
       <c r="C106" s="16" t="str">
         <v>BAJO</v>
       </c>
       <c r="D106" s="17" t="str">
-        <v>Travesaño trasero inferior</v>
+        <v>Lateral</v>
       </c>
       <c r="E106" s="16" t="str">
         <v>RH15 Cartagena</v>
       </c>
       <c r="F106" s="16" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G106" s="16" t="n">
-        <v>490</v>
+        <v>470</v>
       </c>
       <c r="H106" s="16" t="n">
-        <v>80</v>
+        <v>450</v>
       </c>
       <c r="I106" s="16" t="str">
         <v>F</v>
@@ -5594,16 +5594,16 @@
         <v>F</v>
       </c>
       <c r="M106" s="16" t="str">
-        <v>Pequeña</v>
+        <v>Normal</v>
       </c>
       <c r="N106" s="16" t="str">
-        <v>490 × 80</v>
+        <v>470 × 450</v>
       </c>
       <c r="O106" s="16" t="str">
-        <v>489,1 × 79,1</v>
+        <v>469,1 × 449,1</v>
       </c>
       <c r="P106" s="17" t="str">
-        <v>Si no la cantean: cortar a 489.1 × 79.1 y cantear en taller. Zona húmeda: proteger todos los bordes y sellar perforaciones; dimensiones terminadas. Define rigidez posterior; anclajes y uniones por dimensionar. Canto flexible 0,45 mm en todo el perímetro; mantener sellados recortes y perforaciones.</v>
+        <v>Zona húmeda: proteger todos los bordes y sellar perforaciones; dimensiones terminadas. Canto flexible 0,45 mm en todo el perímetro; mantener sellados recortes y perforaciones.</v>
       </c>
     </row>
     <row r="107" ht="100.80000305175781">
@@ -5611,13 +5611,13 @@
         <v>Baño</v>
       </c>
       <c r="B107" s="16" t="str">
-        <v>B06</v>
+        <v>B02</v>
       </c>
       <c r="C107" s="16" t="str">
         <v>BAJO</v>
       </c>
       <c r="D107" s="17" t="str">
-        <v>Panel común para dos puertas: corte diagonal en armado</v>
+        <v>Piso</v>
       </c>
       <c r="E107" s="16" t="str">
         <v>RH15 Cartagena</v>
@@ -5626,34 +5626,34 @@
         <v>1</v>
       </c>
       <c r="G107" s="16" t="n">
-        <v>299</v>
+        <v>490</v>
       </c>
       <c r="H107" s="16" t="n">
-        <v>517</v>
+        <v>450</v>
       </c>
       <c r="I107" s="16" t="str">
-        <v>R</v>
+        <v>F</v>
       </c>
       <c r="J107" s="16" t="str">
-        <v>R</v>
+        <v>F</v>
       </c>
       <c r="K107" s="16" t="str">
-        <v>R</v>
+        <v>F</v>
       </c>
       <c r="L107" s="16" t="str">
-        <v>R</v>
+        <v>F</v>
       </c>
       <c r="M107" s="16" t="str">
         <v>Normal</v>
       </c>
       <c r="N107" s="16" t="str">
-        <v>299 × 517</v>
+        <v>490 × 450</v>
       </c>
       <c r="O107" s="16" t="str">
-        <v>295 × 513</v>
+        <v>489,1 × 449,1</v>
       </c>
       <c r="P107" s="17" t="str">
-        <v>Una sola pieza rectangular terminada 517 × 299 mm (veta vertical). Pedirla entera, con canto 2 mm en el perímetro; NO dividir en tienda. En el armado, corte central a 75° de la horizontal (provisional entre 70 y 80°) con el disco Diablo de 1,5 mm (corte de 0,059") y canto flexible 0,45 mm en los dos bordes nuevos. Holgura entre puertas tras cantear ≈0,6 mm: probablemente insuficiente (ver Pendientes). La medida de lista es del panel común, no de cada tapa.</v>
+        <v>Zona húmeda: proteger todos los bordes y sellar perforaciones; dimensiones terminadas. Canto flexible 0,45 mm en todo el perímetro; mantener sellados recortes y perforaciones.</v>
       </c>
     </row>
     <row r="108" ht="43.20000076293945">
@@ -5661,25 +5661,25 @@
         <v>Baño</v>
       </c>
       <c r="B108" s="16" t="str">
-        <v>S01</v>
+        <v>B03</v>
       </c>
       <c r="C108" s="16" t="str">
-        <v>ESPEJO</v>
+        <v>BAJO</v>
       </c>
       <c r="D108" s="17" t="str">
-        <v>Lateral gabinete superior</v>
+        <v>Entrepaño retranqueado con reserva de sifón</v>
       </c>
       <c r="E108" s="16" t="str">
         <v>RH15 Cartagena</v>
       </c>
       <c r="F108" s="16" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G108" s="16" t="n">
-        <v>500</v>
+        <v>490</v>
       </c>
       <c r="H108" s="16" t="n">
-        <v>105</v>
+        <v>405</v>
       </c>
       <c r="I108" s="16" t="str">
         <v>F</v>
@@ -5697,13 +5697,13 @@
         <v>Normal</v>
       </c>
       <c r="N108" s="16" t="str">
-        <v>500 × 105</v>
+        <v>490 × 405</v>
       </c>
       <c r="O108" s="16" t="str">
-        <v>499,1 × 104,1</v>
+        <v>489,1 × 404,1</v>
       </c>
       <c r="P108" s="17" t="str">
-        <v>Zona húmeda: proteger todos los bordes y sellar perforaciones; dimensiones terminadas. Fondo total 130 mm con panel 6 mm, holgura frontal 1 mm, tapa RH15 y espejo 3 mm. Canto flexible 0,45 mm en todo el perímetro; mantener sellados recortes y perforaciones.</v>
+        <v>Zona húmeda: proteger todos los bordes y sellar perforaciones; dimensiones terminadas. Nicho libre de 150 mm bajo granito. Recorte trasero ilustrativo 100 × 270 mm, centrado; no mecanizar sin sifón real. Retranqueo frontal de 30 mm para agarre. Canto flexible 0,45 mm en todo el perímetro; mantener sellados recortes y perforaciones.</v>
       </c>
     </row>
     <row r="109" ht="28.799999237060547">
@@ -5711,13 +5711,13 @@
         <v>Baño</v>
       </c>
       <c r="B109" s="16" t="str">
-        <v>S02</v>
+        <v>B04</v>
       </c>
       <c r="C109" s="16" t="str">
-        <v>ESPEJO</v>
+        <v>BAJO</v>
       </c>
       <c r="D109" s="17" t="str">
-        <v>Piso y techo gabinete superior</v>
+        <v>Travesaño trasero superior lateral</v>
       </c>
       <c r="E109" s="16" t="str">
         <v>RH15 Cartagena</v>
@@ -5726,10 +5726,10 @@
         <v>2</v>
       </c>
       <c r="G109" s="16" t="n">
-        <v>420</v>
+        <v>195</v>
       </c>
       <c r="H109" s="16" t="n">
-        <v>105</v>
+        <v>80</v>
       </c>
       <c r="I109" s="16" t="str">
         <v>F</v>
@@ -5744,16 +5744,16 @@
         <v>F</v>
       </c>
       <c r="M109" s="16" t="str">
-        <v>Normal</v>
+        <v>Pequeña</v>
       </c>
       <c r="N109" s="16" t="str">
-        <v>420 × 105</v>
+        <v>195 × 80</v>
       </c>
       <c r="O109" s="16" t="str">
-        <v>419,1 × 104,1</v>
+        <v>194,1 × 79,1</v>
       </c>
       <c r="P109" s="17" t="str">
-        <v>Zona húmeda: proteger todos los bordes y sellar perforaciones; dimensiones terminadas. Canto flexible 0,45 mm en todo el perímetro; mantener sellados recortes y perforaciones.</v>
+        <v>Si no la cantean: cortar a 194.1 × 79.1 y cantear en taller. Zona húmeda: proteger todos los bordes y sellar perforaciones; dimensiones terminadas. De canto, interrumpido en el centro para tuberías; no es un colgador certificado. Canto flexible 0,45 mm en todo el perímetro; mantener sellados recortes y perforaciones.</v>
       </c>
     </row>
     <row r="110" ht="43.20000076293945">
@@ -5761,13 +5761,13 @@
         <v>Baño</v>
       </c>
       <c r="B110" s="16" t="str">
-        <v>S03</v>
+        <v>B05</v>
       </c>
       <c r="C110" s="16" t="str">
-        <v>ESPEJO</v>
+        <v>BAJO</v>
       </c>
       <c r="D110" s="17" t="str">
-        <v>División vertical</v>
+        <v>Travesaño trasero inferior</v>
       </c>
       <c r="E110" s="16" t="str">
         <v>RH15 Cartagena</v>
@@ -5776,10 +5776,10 @@
         <v>1</v>
       </c>
       <c r="G110" s="16" t="n">
-        <v>470</v>
+        <v>490</v>
       </c>
       <c r="H110" s="16" t="n">
-        <v>105</v>
+        <v>80</v>
       </c>
       <c r="I110" s="16" t="str">
         <v>F</v>
@@ -5794,16 +5794,16 @@
         <v>F</v>
       </c>
       <c r="M110" s="16" t="str">
-        <v>Normal</v>
+        <v>Pequeña</v>
       </c>
       <c r="N110" s="16" t="str">
-        <v>470 × 105</v>
+        <v>490 × 80</v>
       </c>
       <c r="O110" s="16" t="str">
-        <v>469,1 × 104,1</v>
+        <v>489,1 × 79,1</v>
       </c>
       <c r="P110" s="17" t="str">
-        <v>Zona húmeda: proteger todos los bordes y sellar perforaciones; dimensiones terminadas. Interior cerrado 290 mm; columna derecha abierta 115 mm. Canto flexible 0,45 mm en todo el perímetro; mantener sellados recortes y perforaciones.</v>
+        <v>Si no la cantean: cortar a 489.1 × 79.1 y cantear en taller. Zona húmeda: proteger todos los bordes y sellar perforaciones; dimensiones terminadas. Define rigidez posterior; anclajes y uniones por dimensionar. Canto flexible 0,45 mm en todo el perímetro; mantener sellados recortes y perforaciones.</v>
       </c>
     </row>
     <row r="111" ht="43.20000076293945">
@@ -5811,49 +5811,49 @@
         <v>Baño</v>
       </c>
       <c r="B111" s="16" t="str">
-        <v>S04</v>
+        <v>B06</v>
       </c>
       <c r="C111" s="16" t="str">
-        <v>ESPEJO</v>
+        <v>BAJO</v>
       </c>
       <c r="D111" s="17" t="str">
-        <v>Entrepaño interior izquierdo</v>
+        <v>Panel común para dos puertas: corte diagonal en armado</v>
       </c>
       <c r="E111" s="16" t="str">
         <v>RH15 Cartagena</v>
       </c>
       <c r="F111" s="16" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G111" s="16" t="n">
-        <v>290</v>
+        <v>299</v>
       </c>
       <c r="H111" s="16" t="n">
-        <v>100</v>
+        <v>517</v>
       </c>
       <c r="I111" s="16" t="str">
-        <v>F</v>
+        <v>R</v>
       </c>
       <c r="J111" s="16" t="str">
-        <v>F</v>
+        <v>R</v>
       </c>
       <c r="K111" s="16" t="str">
-        <v>F</v>
+        <v>R</v>
       </c>
       <c r="L111" s="16" t="str">
-        <v>F</v>
+        <v>R</v>
       </c>
       <c r="M111" s="16" t="str">
-        <v>Pequeña</v>
+        <v>Normal</v>
       </c>
       <c r="N111" s="16" t="str">
-        <v>290 × 100</v>
+        <v>299 × 517</v>
       </c>
       <c r="O111" s="16" t="str">
-        <v>289,1 × 99,1</v>
+        <v>295 × 513</v>
       </c>
       <c r="P111" s="17" t="str">
-        <v>Si no la cantean: cortar a 289.1 × 99.1 y cantear en taller. Zona húmeda: proteger todos los bordes y sellar perforaciones; dimensiones terminadas. Dos entrepaños fijos como la referencia. Canto flexible 0,45 mm en todo el perímetro; mantener sellados recortes y perforaciones.</v>
+        <v>Una sola pieza rectangular terminada 517 × 299 mm (veta vertical). Pedirla entera, con canto 2 mm en el perímetro; NO dividir en tienda. En el armado, corte central a 75° de la horizontal (provisional entre 70 y 80°) con el disco Diablo de 1,5 mm (corte de 0,059") y canto flexible 0,45 mm en los dos bordes nuevos. Holgura entre puertas tras cantear ≈0,6 mm: probablemente insuficiente (ver Pendientes). La medida de lista es del panel común, no de cada tapa.</v>
       </c>
     </row>
     <row r="112" ht="43.20000076293945">
@@ -5861,25 +5861,25 @@
         <v>Baño</v>
       </c>
       <c r="B112" s="16" t="str">
-        <v>S05</v>
+        <v>S01</v>
       </c>
       <c r="C112" s="16" t="str">
         <v>ESPEJO</v>
       </c>
       <c r="D112" s="17" t="str">
-        <v>Entrepaño columna abierta derecha</v>
+        <v>Lateral gabinete superior</v>
       </c>
       <c r="E112" s="16" t="str">
         <v>RH15 Cartagena</v>
       </c>
       <c r="F112" s="16" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G112" s="16" t="n">
-        <v>115</v>
+        <v>500</v>
       </c>
       <c r="H112" s="16" t="n">
-        <v>100</v>
+        <v>105</v>
       </c>
       <c r="I112" s="16" t="str">
         <v>F</v>
@@ -5894,16 +5894,16 @@
         <v>F</v>
       </c>
       <c r="M112" s="16" t="str">
-        <v>Pequeña</v>
+        <v>Normal</v>
       </c>
       <c r="N112" s="16" t="str">
-        <v>115 × 100</v>
+        <v>500 × 105</v>
       </c>
       <c r="O112" s="16" t="str">
-        <v>114,1 × 99,1</v>
+        <v>499,1 × 104,1</v>
       </c>
       <c r="P112" s="17" t="str">
-        <v>Si no la cantean: cortar a 114.1 × 99.1 y cantear en taller. Zona húmeda: proteger todos los bordes y sellar perforaciones; dimensiones terminadas. Canto flexible 0,45 mm en todo el perímetro; mantener sellados recortes y perforaciones.</v>
+        <v>Zona húmeda: proteger todos los bordes y sellar perforaciones; dimensiones terminadas. Fondo total 130 mm con panel 6 mm, holgura frontal 1 mm, tapa RH15 y espejo 3 mm. Canto flexible 0,45 mm en todo el perímetro; mantener sellados recortes y perforaciones.</v>
       </c>
     </row>
     <row r="113" ht="43.20000076293945">
@@ -5911,25 +5911,25 @@
         <v>Baño</v>
       </c>
       <c r="B113" s="16" t="str">
-        <v>S06</v>
+        <v>S02</v>
       </c>
       <c r="C113" s="16" t="str">
         <v>ESPEJO</v>
       </c>
       <c r="D113" s="17" t="str">
-        <v>Tapa RH15 portadora del espejo</v>
+        <v>Piso y techo gabinete superior</v>
       </c>
       <c r="E113" s="16" t="str">
         <v>RH15 Cartagena</v>
       </c>
       <c r="F113" s="16" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G113" s="16" t="n">
-        <v>500</v>
+        <v>420</v>
       </c>
       <c r="H113" s="16" t="n">
-        <v>320</v>
+        <v>105</v>
       </c>
       <c r="I113" s="16" t="str">
         <v>F</v>
@@ -5947,13 +5947,13 @@
         <v>Normal</v>
       </c>
       <c r="N113" s="16" t="str">
-        <v>500 × 320</v>
+        <v>420 × 105</v>
       </c>
       <c r="O113" s="16" t="str">
-        <v>499,1 × 319,1</v>
+        <v>419,1 × 104,1</v>
       </c>
       <c r="P113" s="17" t="str">
-        <v>Medida exterior de referencia 320 × 500; espejo pegado en cara exterior. Dos bisagras candidatas, peso conjunto aproximado 2,8 kg sin herrajes. Validar holguras, cazoletas y adhesivo compatible con espejo. Canto flexible 0,45 mm en todo el perímetro; mantener sellados recortes y perforaciones.</v>
+        <v>Zona húmeda: proteger todos los bordes y sellar perforaciones; dimensiones terminadas. Canto flexible 0,45 mm en todo el perímetro; mantener sellados recortes y perforaciones.</v>
       </c>
     </row>
     <row r="114" ht="43.20000076293945">
@@ -5961,25 +5961,25 @@
         <v>Baño</v>
       </c>
       <c r="B114" s="16" t="str">
-        <v>F01</v>
+        <v>S03</v>
       </c>
       <c r="C114" s="16" t="str">
         <v>ESPEJO</v>
       </c>
       <c r="D114" s="17" t="str">
-        <v>Fondo blanco de 6 mm</v>
+        <v>División vertical</v>
       </c>
       <c r="E114" s="16" t="str">
-        <v>Fondo melamina blanco RH6</v>
+        <v>RH15 Cartagena</v>
       </c>
       <c r="F114" s="16" t="n">
         <v>1</v>
       </c>
       <c r="G114" s="16" t="n">
-        <v>496</v>
+        <v>470</v>
       </c>
       <c r="H114" s="16" t="n">
-        <v>446</v>
+        <v>105</v>
       </c>
       <c r="I114" s="16" t="str">
         <v>F</v>
@@ -5997,17 +5997,217 @@
         <v>Normal</v>
       </c>
       <c r="N114" s="16" t="str">
+        <v>470 × 105</v>
+      </c>
+      <c r="O114" s="16" t="str">
+        <v>469,1 × 104,1</v>
+      </c>
+      <c r="P114" s="17" t="str">
+        <v>Zona húmeda: proteger todos los bordes y sellar perforaciones; dimensiones terminadas. Interior cerrado 290 mm; columna derecha abierta 115 mm. Canto flexible 0,45 mm en todo el perímetro; mantener sellados recortes y perforaciones.</v>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" s="13" t="str">
+        <v>Baño</v>
+      </c>
+      <c r="B115" s="13" t="str">
+        <v>S04</v>
+      </c>
+      <c r="C115" s="13" t="str">
+        <v>ESPEJO</v>
+      </c>
+      <c r="D115" s="13" t="str">
+        <v>Entrepaño interior izquierdo</v>
+      </c>
+      <c r="E115" s="13" t="str">
+        <v>RH15 Cartagena</v>
+      </c>
+      <c r="F115" s="13" t="n">
+        <v>2</v>
+      </c>
+      <c r="G115" s="13" t="n">
+        <v>290</v>
+      </c>
+      <c r="H115" s="13" t="n">
+        <v>100</v>
+      </c>
+      <c r="I115" s="13" t="str">
+        <v>F</v>
+      </c>
+      <c r="J115" s="13" t="str">
+        <v>F</v>
+      </c>
+      <c r="K115" s="13" t="str">
+        <v>F</v>
+      </c>
+      <c r="L115" s="13" t="str">
+        <v>F</v>
+      </c>
+      <c r="M115" s="13" t="str">
+        <v>Pequeña</v>
+      </c>
+      <c r="N115" s="13" t="str">
+        <v>290 × 100</v>
+      </c>
+      <c r="O115" s="13" t="str">
+        <v>289,1 × 99,1</v>
+      </c>
+      <c r="P115" s="13" t="str">
+        <v>Si no la cantean: cortar a 289.1 × 99.1 y cantear en taller. Zona húmeda: proteger todos los bordes y sellar perforaciones; dimensiones terminadas. Dos entrepaños fijos como la referencia. Canto flexible 0,45 mm en todo el perímetro; mantener sellados recortes y perforaciones.</v>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" s="13" t="str">
+        <v>Baño</v>
+      </c>
+      <c r="B116" s="13" t="str">
+        <v>S05</v>
+      </c>
+      <c r="C116" s="13" t="str">
+        <v>ESPEJO</v>
+      </c>
+      <c r="D116" s="13" t="str">
+        <v>Entrepaño columna abierta derecha</v>
+      </c>
+      <c r="E116" s="13" t="str">
+        <v>RH15 Cartagena</v>
+      </c>
+      <c r="F116" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="G116" s="13" t="n">
+        <v>115</v>
+      </c>
+      <c r="H116" s="13" t="n">
+        <v>100</v>
+      </c>
+      <c r="I116" s="13" t="str">
+        <v>F</v>
+      </c>
+      <c r="J116" s="13" t="str">
+        <v>F</v>
+      </c>
+      <c r="K116" s="13" t="str">
+        <v>F</v>
+      </c>
+      <c r="L116" s="13" t="str">
+        <v>F</v>
+      </c>
+      <c r="M116" s="13" t="str">
+        <v>Pequeña</v>
+      </c>
+      <c r="N116" s="13" t="str">
+        <v>115 × 100</v>
+      </c>
+      <c r="O116" s="13" t="str">
+        <v>114,1 × 99,1</v>
+      </c>
+      <c r="P116" s="13" t="str">
+        <v>Si no la cantean: cortar a 114.1 × 99.1 y cantear en taller. Zona húmeda: proteger todos los bordes y sellar perforaciones; dimensiones terminadas. Canto flexible 0,45 mm en todo el perímetro; mantener sellados recortes y perforaciones.</v>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" s="13" t="str">
+        <v>Baño</v>
+      </c>
+      <c r="B117" s="13" t="str">
+        <v>S06</v>
+      </c>
+      <c r="C117" s="13" t="str">
+        <v>ESPEJO</v>
+      </c>
+      <c r="D117" s="13" t="str">
+        <v>Tapa RH15 portadora del espejo</v>
+      </c>
+      <c r="E117" s="13" t="str">
+        <v>RH15 Cartagena</v>
+      </c>
+      <c r="F117" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="G117" s="13" t="n">
+        <v>500</v>
+      </c>
+      <c r="H117" s="13" t="n">
+        <v>320</v>
+      </c>
+      <c r="I117" s="13" t="str">
+        <v>F</v>
+      </c>
+      <c r="J117" s="13" t="str">
+        <v>F</v>
+      </c>
+      <c r="K117" s="13" t="str">
+        <v>F</v>
+      </c>
+      <c r="L117" s="13" t="str">
+        <v>F</v>
+      </c>
+      <c r="M117" s="13" t="str">
+        <v>Normal</v>
+      </c>
+      <c r="N117" s="13" t="str">
+        <v>500 × 320</v>
+      </c>
+      <c r="O117" s="13" t="str">
+        <v>499,1 × 319,1</v>
+      </c>
+      <c r="P117" s="13" t="str">
+        <v>Medida exterior de referencia 320 × 500; espejo pegado en cara exterior. Dos bisagras candidatas, peso conjunto aproximado 2,8 kg sin herrajes. Validar holguras, cazoletas y adhesivo compatible con espejo. Canto flexible 0,45 mm en todo el perímetro; mantener sellados recortes y perforaciones.</v>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" s="13" t="str">
+        <v>Baño</v>
+      </c>
+      <c r="B118" s="13" t="str">
+        <v>F01</v>
+      </c>
+      <c r="C118" s="13" t="str">
+        <v>ESPEJO</v>
+      </c>
+      <c r="D118" s="13" t="str">
+        <v>Fondo blanco de 6 mm</v>
+      </c>
+      <c r="E118" s="13" t="str">
+        <v>Fondo melamina blanco RH6</v>
+      </c>
+      <c r="F118" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="G118" s="13" t="n">
+        <v>496</v>
+      </c>
+      <c r="H118" s="13" t="n">
+        <v>446</v>
+      </c>
+      <c r="I118" s="13" t="str">
+        <v>F</v>
+      </c>
+      <c r="J118" s="13" t="str">
+        <v>F</v>
+      </c>
+      <c r="K118" s="13" t="str">
+        <v>F</v>
+      </c>
+      <c r="L118" s="13" t="str">
+        <v>F</v>
+      </c>
+      <c r="M118" s="13" t="str">
+        <v>Normal</v>
+      </c>
+      <c r="N118" s="13" t="str">
         <v>496 × 446</v>
       </c>
-      <c r="O114" s="16" t="str">
+      <c r="O118" s="13" t="str">
         <v>495,1 × 445,1</v>
       </c>
-      <c r="P114" s="17" t="str">
+      <c r="P118" s="13" t="str">
         <v>Fondo aplicado por detrás, retranqueado 2 mm de los bordes. Reutilización de sobrantes de cocina solo se comprobará en la optimización conjunta final. No soporta el anclaje del gabinete. Canto flexible 0,45 mm en todo el perímetro; mantener sellados recortes y perforaciones.</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A6:P114"/>
+  <autoFilter ref="A6:P118"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -6029,7 +6229,7 @@
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="11" t="str">
-        <x:v>Cortes pasantes, sin rotar por la veta, refilado 10 mm por lado y sierra 4 mm. El plano de corte definitivo lo define la seccionadora del proveedor.</x:v>
+        <x:v>Cortes pasantes, sin rotar por la veta, refilado 10 mm por lado y sierra 5 mm. El plano de corte definitivo lo define la seccionadora del proveedor.</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
@@ -6054,10 +6254,10 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="C7" s="18" t="n">
-        <x:v>0.969</x:v>
+        <x:v>0.954</x:v>
       </x:c>
       <x:c r="D7" s="17" t="str">
-        <x:v>Clóset C3-011, Clóset C3-023, Cocina P016, Cocina P011, Cocina P002, Cocina P019, Cocina P019, Cocina P018, Cocina P003, Cocina P003</x:v>
+        <x:v>Clóset C3-023, Clóset C3-023, Clóset C3-024, Cocina P016, Cocina P011, Cocina P040, Cocina P043, Clóset C3-019, Clóset C3-019, Baño B04, Baño B04, Cocina P003, Cocina P003</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="28.799999237060547">
@@ -6068,10 +6268,10 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="C8" s="18" t="n">
-        <x:v>0.886</x:v>
+        <x:v>0.928</x:v>
       </x:c>
       <x:c r="D8" s="17" t="str">
-        <x:v>Clóset C3-023, Clóset C3-009, Clóset C3-010, Clóset C3-012, Clóset C3-006, Clóset C3-020, Cocina P040, Cocina P041, Cocina P043, Clóset C3-019, Baño B04, Baño S05</x:v>
+        <x:v>Clóset C3-001, Clóset C3-001, Clóset C3-002, Clóset C3-010, Clóset C3-012, Cocina P041, Baño S05</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -6082,10 +6282,10 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="C9" s="18" t="n">
-        <x:v>0.89</x:v>
+        <x:v>0.924</x:v>
       </x:c>
       <x:c r="D9" s="17" t="str">
-        <x:v>Clóset C3-005, Cocina P037, Clóset C3-003, Cocina P001, Cocina P001, Cocina P024, Baño B02, Clóset C3-021, Baño S03, Baño B04</x:v>
+        <x:v>Clóset C3-009, Cocina P037, Clóset C3-003, Cocina P001, Cocina P001, Cocina P006, Cocina P024, Cocina P013, Cocina P070, Cocina P063, Cocina P064, Baño B02, Baño S01</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
@@ -6096,10 +6296,10 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="C10" s="18" t="n">
-        <x:v>0.895</x:v>
+        <x:v>0.934</x:v>
       </x:c>
       <x:c r="D10" s="17" t="str">
-        <x:v>Clóset C3-001, Clóset C3-001, Cocina P006, Cocina P006, Cocina P013, Cocina P070, Cocina P063, Cocina P064</x:v>
+        <x:v>Cocina P006, Cocina P012, Cocina P012, Cocina P023, Cocina P023, Cocina P030, Cocina P030, Clóset C3-004, Clóset C3-017, Cocina P022, Cocina P027, Cocina P028</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
@@ -6110,10 +6310,10 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="C11" s="18" t="n">
-        <x:v>0.885</x:v>
+        <x:v>0.883</x:v>
       </x:c>
       <x:c r="D11" s="17" t="str">
-        <x:v>Clóset C3-002, Cocina P012, Cocina P012, Cocina P023, Cocina P023, Clóset C3-017, Clóset C3-017, Cocina P022, Cocina P029, Baño B01</x:v>
+        <x:v>Clóset C3-006, Clóset C3-017, Clóset C3-017, Cocina P029, Cocina P017, Cocina P007, Cocina P009, Cocina P056, Cocina P057, Cocina P039, Cocina P039, Cocina P050, Cocina P050, Cocina P058, Cocina P031, Cocina P002, Cocina P025, Cocina P008, Cocina P061, Cocina P010, Cocina P018</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="43.20000076293945">
@@ -6124,10 +6324,10 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="C12" s="18" t="n">
-        <x:v>0.909</x:v>
+        <x:v>0.784</x:v>
       </x:c>
       <x:c r="D12" s="17" t="str">
-        <x:v>Cocina P030, Cocina P030, Clóset C3-004, Clóset C3-017, Cocina P017, Cocina P009, Cocina P027, Cocina P028, Clóset C3-024, Cocina P056, Cocina P057, Cocina P039, Cocina P039, Cocina P038, Cocina P066, Clóset C3-014, Clóset C3-013, Clóset C3-007, Baño S02, Cocina P060, Baño B05, Clóset C3-019, Clóset C3-019, Baño S04, Baño S04</x:v>
+        <x:v>Cocina P058, Cocina P065, Cocina P065, Cocina P059, Cocina P054, Baño B01, Baño B01, Cocina P049, Cocina P034, Cocina P051, Cocina P052, Baño B03, Cocina P046, Cocina P047, Cocina P020, Cocina P035, Baño B06, Cocina P036, Cocina P055, Cocina P055, Clóset C3-016, Clóset C3-016, Clóset C3-016, Baño S01, Baño S03, Baño S04, Baño S04</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="43.20000076293945">
@@ -6138,10 +6338,10 @@
         <x:v>7</x:v>
       </x:c>
       <x:c r="C13" s="18" t="n">
-        <x:v>0.897</x:v>
+        <x:v>0.75</x:v>
       </x:c>
       <x:c r="D13" s="17" t="str">
-        <x:v>Cocina P007, Cocina P050, Cocina P050, Cocina P058, Cocina P058, Cocina P065, Cocina P065, Cocina P059, Cocina P031, Cocina P054, Baño B01, Cocina P051, Cocina P052, Clóset C3-015, Clóset C3-015, Clóset C3-015, Cocina P044, Cocina P005, Cocina P038, Cocina P067, Cocina P045, Cocina P055, Cocina P055, Clóset C3-008, Cocina P025, Cocina P025, Cocina P014, Cocina P014, Cocina P061</x:v>
+        <x:v>Clóset C3-027, Clóset C3-028, Clóset C3-020, Cocina P021, Clóset C3-015, Clóset C3-015, Clóset C3-015, Baño S06, Cocina P044, Cocina P005, Cocina P038, Cocina P038, Clóset C3-018, Clóset C3-018, Clóset C3-018, Clóset C3-018, Clóset C3-018, Clóset C3-018, Cocina P066, Cocina P067, Cocina P045, Cocina P045, Cocina P069, Clóset C3-016, Clóset C3-016, Clóset C3-016, Cocina P025, Cocina P014, Cocina P014, Baño S02, Baño S02, Cocina P019, Cocina P019, Cocina P032, Cocina P032</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="57.599998474121094">
@@ -6152,10 +6352,10 @@
         <x:v>8</x:v>
       </x:c>
       <x:c r="C14" s="18" t="n">
-        <x:v>0.731</x:v>
+        <x:v>0.228</x:v>
       </x:c>
       <x:c r="D14" s="17" t="str">
-        <x:v>Cocina P049, Cocina P034, Baño B03, Cocina P046, Cocina P047, Cocina P020, Cocina P021, Baño S06, Cocina P035, Baño B06, Clóset C3-018, Clóset C3-018, Clóset C3-018, Clóset C3-018, Clóset C3-018, Clóset C3-018, Cocina P036, Cocina P045, Cocina P069, Clóset C3-016, Clóset C3-016, Clóset C3-016, Clóset C3-016, Clóset C3-016, Clóset C3-016, Cocina P008, Baño S01, Baño S01, Cocina P010, Baño S02, Cocina P018, Clóset C3-022, Clóset C3-022, Clóset C3-022, Cocina P032, Cocina P032, Cocina P071</x:v>
+        <x:v>Clóset C3-021, Clóset C3-026, Clóset C3-014, Clóset C3-030, Clóset C3-013, Clóset C3-025, Clóset C3-008, Clóset C3-029, Clóset C3-007, Cocina P018, Cocina P060, Baño B05, Clóset C3-022, Clóset C3-022, Clóset C3-022, Cocina P071, Clóset C3-019</x:v>
       </x:c>
     </x:row>
     <x:row r="15">
@@ -6289,10 +6489,10 @@
         <x:v>Clóset</x:v>
       </x:c>
       <x:c r="C13" s="13" t="n">
-        <x:v>51.885</x:v>
+        <x:v>59.795</x:v>
       </x:c>
       <x:c r="D13" s="13" t="n">
-        <x:v>80</x:v>
+        <x:v>86</x:v>
       </x:c>
     </x:row>
     <x:row r="14">
@@ -6314,13 +6514,13 @@
         <x:v>Flexible 0,45 mm</x:v>
       </x:c>
       <x:c r="B15" s="14" t="str">
-        <x:v>Total · comprar 172 m</x:v>
+        <x:v>Total · comprar 181 m</x:v>
       </x:c>
       <x:c r="C15" s="14" t="n">
-        <x:v>141.296</x:v>
+        <x:v>149.206</x:v>
       </x:c>
       <x:c r="D15" s="14" t="n">
-        <x:v>300</x:v>
+        <x:v>306</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -6402,7 +6602,7 @@
         <x:v>2926976</x:v>
       </x:c>
       <x:c r="H10" s="17" t="str">
-        <x:v>Encaje conjunto de las piezas RH15 de los tres muebles en 8 láminas (hoja Láminas). Por separado serían 10.</x:v>
+        <x:v>Encaje conjunto de las piezas RH15 de los tres muebles en 8 láminas (hoja Láminas). Por separado serían 9.</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
@@ -6510,7 +6710,7 @@
         <x:v>285600</x:v>
       </x:c>
       <x:c r="H14" s="17" t="str">
-        <x:v>Necesario 172 m: 141,3 m netos + 5 cm por borde (300 bordes) + 10 %. Sobran unos 28 m para cantear en el armado las piezas pequeñas que no acepte la máquina.</x:v>
+        <x:v>Necesario 181 m: 149,2 m netos + 5 cm por borde (306 bordes) + 10 %. Sobran unos 19 m para cantear en el armado las piezas pequeñas que no acepte la máquina.</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="28.799999237060547">
@@ -7090,7 +7290,7 @@
         <x:v>Por cotizar</x:v>
       </x:c>
       <x:c r="H37" s="17" t="str">
-        <x:v>Incluye fijación de fondos, estructura y refuerzos de RH; el bastidor del riel se lista aparte. El extremo derecho queda libre: no puede anclarse al muro lateral derecho. Definir anclaje posterior y lateral izquierdo según muro.</x:v>
+        <x:v>Unir el marco completo C3-025 a C3-030 a laterales, divisor, pisos y tapas. Dimensionar anclajes al muro posterior resistente y al izquierdo. No fijar solo al estuco. El lateral derecho queda libre: el montante se une a la caja y al muro de fondo, no a una pared lateral inexistente. El marco abierto no se da por equivalente a un panel arriostrante.</x:v>
       </x:c>
     </x:row>
     <x:row r="38" ht="72">
@@ -7859,7 +8059,7 @@
         <x:v>Travesaño horizontal</x:v>
       </x:c>
       <x:c r="D8" s="17" t="str">
-        <x:v>Si no la cantean: cortar a 150 × 99.1 y cantear en el armado. Rebaje para la gola en el armado, cuando se defina el borde del granito; no lo hace el proveedor.</x:v>
+        <x:v>Si no la cantean: cortar a 150 × 99,1 y cantear en el armado. Rebaje para la gola en el armado, cuando se defina el borde del granito; no lo hace el proveedor.</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -7915,7 +8115,7 @@
         <x:v>Travesaño horizontal</x:v>
       </x:c>
       <x:c r="D12" s="17" t="str">
-        <x:v>Si no la cantean: cortar a 640 × 99.1 y cantear en el armado. Rebaje para la gola en el armado, cuando se defina el borde del granito; no lo hace el proveedor.</x:v>
+        <x:v>Si no la cantean: cortar a 640 × 99,1 y cantear en el armado. Rebaje para la gola en el armado, cuando se defina el borde del granito; no lo hace el proveedor.</x:v>
       </x:c>
     </x:row>
     <x:row r="13">
@@ -7943,7 +8143,7 @@
         <x:v>Travesaño de canto</x:v>
       </x:c>
       <x:c r="D14" s="17" t="str">
-        <x:v>Si no la cantean: cortar a 669.1 × 99.1 y cantear en el armado. Rebaje para la gola en el armado, cuando se defina el borde del granito; no lo hace el proveedor.</x:v>
+        <x:v>Si no la cantean: cortar a 669,1 × 99,1 y cantear en el armado. Rebaje para la gola en el armado, cuando se defina el borde del granito; no lo hace el proveedor.</x:v>
       </x:c>
     </x:row>
     <x:row r="15">
@@ -7985,7 +8185,7 @@
         <x:v>Travesaño horizontal</x:v>
       </x:c>
       <x:c r="D17" s="17" t="str">
-        <x:v>Si no la cantean: cortar a 370 × 99.1 y cantear en el armado. Rebaje para la gola en el armado, cuando se defina el borde del granito; no lo hace el proveedor.</x:v>
+        <x:v>Si no la cantean: cortar a 370 × 99,1 y cantear en el armado. Rebaje para la gola en el armado, cuando se defina el borde del granito; no lo hace el proveedor.</x:v>
       </x:c>
     </x:row>
     <x:row r="18">
@@ -8027,7 +8227,7 @@
         <x:v>PROVISIONAL larguero bajo plataforma basurero</x:v>
       </x:c>
       <x:c r="D20" s="17" t="str">
-        <x:v>Si no la cantean: cortar a 549.1 × 59.1 y cantear en el armado. NO PEDIR: se corta en el armado de un sobrante, con el riel HRE126-55 y la bandeja en mano. Pedir a la sucursal que entregue los sobrantes.</x:v>
+        <x:v>Si no la cantean: cortar a 549,1 × 59,1 y cantear en el armado. NO PEDIR: se corta en el armado de un sobrante, con el riel HRE126-55 y la bandeja en mano. Pedir a la sucursal que entregue los sobrantes.</x:v>
       </x:c>
     </x:row>
     <x:row r="21" ht="28.799999237060547">
@@ -8041,7 +8241,7 @@
         <x:v>PROVISIONAL travesaño bajo plataforma basurero</x:v>
       </x:c>
       <x:c r="D21" s="17" t="str">
-        <x:v>Si no la cantean: cortar a 312.1 × 59.1 y cantear en el armado. NO PEDIR: se corta en el armado de un sobrante, con el riel HRE126-55 y la bandeja en mano. Pedir a la sucursal que entregue los sobrantes.</x:v>
+        <x:v>Si no la cantean: cortar a 312,1 × 59,1 y cantear en el armado. NO PEDIR: se corta en el armado de un sobrante, con el riel HRE126-55 y la bandeja en mano. Pedir a la sucursal que entregue los sobrantes.</x:v>
       </x:c>
     </x:row>
     <x:row r="22">

</xml_diff>